<commit_message>
depuracion de directorios, archivos y script innecesarios
</commit_message>
<xml_diff>
--- a/results/logs/episode_rewards.xlsx
+++ b/results/logs/episode_rewards.xlsx
@@ -30553,10 +30553,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>26.02730117575042</v>
+        <v>26.02730117575039</v>
       </c>
       <c r="C4" t="n">
-        <v>28.90206609405679</v>
+        <v>28.90206609405676</v>
       </c>
       <c r="D4" t="n">
         <v>152.2214650059671</v>
@@ -30565,7 +30565,7 @@
         <v>9.283984024749472</v>
       </c>
       <c r="F4" t="n">
-        <v>21.02872370862951</v>
+        <v>21.02872370862949</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
ajustes de los parametros del agente de carga
</commit_message>
<xml_diff>
--- a/results/logs/episode_rewards.xlsx
+++ b/results/logs/episode_rewards.xlsx
@@ -478,7 +478,7 @@
         <v>-3.159722222222224</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>8.600000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -563,7 +563,7 @@
         <v>-3.159722222222224</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>8.600000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -597,7 +597,7 @@
         <v>-3.159722222222224</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>8.600000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -619,7 +619,7 @@
         <v>-3.159722222222224</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>8.600000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -641,7 +641,7 @@
         <v>-3.159722222222224</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>8.600000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -663,7 +663,7 @@
         <v>-3.159722222222224</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>8.600000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -685,7 +685,7 @@
         <v>-3.159722222222224</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>8.600000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
se ajusto los nuevos idx
</commit_message>
<xml_diff>
--- a/results/logs/episode_rewards.xlsx
+++ b/results/logs/episode_rewards.xlsx
@@ -472,10 +472,10 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>-3.5</v>
       </c>
       <c r="E2" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
         <v>7</v>
@@ -557,10 +557,10 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>8</v>
+        <v>-3.5</v>
       </c>
       <c r="E3" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
         <v>7</v>
@@ -591,10 +591,10 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>8</v>
+        <v>-3.5</v>
       </c>
       <c r="E5" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
         <v>7</v>
@@ -613,10 +613,10 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>-3.5</v>
       </c>
       <c r="E6" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
         <v>7</v>
@@ -635,10 +635,10 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>8</v>
+        <v>-3.5</v>
       </c>
       <c r="E7" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
         <v>7</v>
@@ -657,10 +657,10 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>8</v>
+        <v>-3.5</v>
       </c>
       <c r="E8" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
         <v>7</v>
@@ -679,10 +679,10 @@
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>-3.5</v>
       </c>
       <c r="E9" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
         <v>7</v>

</xml_diff>

<commit_message>
caso de estudio 2 ok OJO
</commit_message>
<xml_diff>
--- a/results/logs/episode_rewards.xlsx
+++ b/results/logs/episode_rewards.xlsx
@@ -9358,7 +9358,7 @@
         <v>11.5</v>
       </c>
       <c r="F446" t="n">
-        <v>11.5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="447">
@@ -9838,7 +9838,7 @@
         <v>24.5</v>
       </c>
       <c r="F470" t="n">
-        <v>20.5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="471">
@@ -10058,7 +10058,7 @@
         <v>32.5</v>
       </c>
       <c r="F481" t="n">
-        <v>14.5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="482">
@@ -11118,7 +11118,7 @@
         <v>-12</v>
       </c>
       <c r="F534" t="n">
-        <v>19</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="535">
@@ -12398,7 +12398,7 @@
         <v>13.75</v>
       </c>
       <c r="F598" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="599">
@@ -12498,7 +12498,7 @@
         <v>26.5</v>
       </c>
       <c r="F603" t="n">
-        <v>17.5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="604">
@@ -14058,7 +14058,7 @@
         <v>11</v>
       </c>
       <c r="F681" t="n">
-        <v>13</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="682">
@@ -14078,7 +14078,7 @@
         <v>22</v>
       </c>
       <c r="F682" t="n">
-        <v>14.5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="683">
@@ -14098,7 +14098,7 @@
         <v>11.25</v>
       </c>
       <c r="F683" t="n">
-        <v>16</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="684">
@@ -14278,7 +14278,7 @@
         <v>37.75</v>
       </c>
       <c r="F692" t="n">
-        <v>20.5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="693">
@@ -14458,7 +14458,7 @@
         <v>37</v>
       </c>
       <c r="F701" t="n">
-        <v>22</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="702">
@@ -14478,7 +14478,7 @@
         <v>13</v>
       </c>
       <c r="F702" t="n">
-        <v>19</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="703">
@@ -15038,7 +15038,7 @@
         <v>6</v>
       </c>
       <c r="F730" t="n">
-        <v>5.5</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="731">
@@ -15618,7 +15618,7 @@
         <v>-4</v>
       </c>
       <c r="F759" t="n">
-        <v>16</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="760">
@@ -15638,7 +15638,7 @@
         <v>-4.75</v>
       </c>
       <c r="F760" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="761">
@@ -15678,7 +15678,7 @@
         <v>33</v>
       </c>
       <c r="F762" t="n">
-        <v>17.5</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="763">
@@ -16298,7 +16298,7 @@
         <v>36</v>
       </c>
       <c r="F793" t="n">
-        <v>17.5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="794">
@@ -16978,7 +16978,7 @@
         <v>-7.5</v>
       </c>
       <c r="F827" t="n">
-        <v>17.5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="828">
@@ -16998,7 +16998,7 @@
         <v>31.25</v>
       </c>
       <c r="F828" t="n">
-        <v>14.5</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="829">
@@ -17358,7 +17358,7 @@
         <v>-1.25</v>
       </c>
       <c r="F846" t="n">
-        <v>14.5</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="847">
@@ -17398,7 +17398,7 @@
         <v>25</v>
       </c>
       <c r="F848" t="n">
-        <v>22</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="849">
@@ -17418,7 +17418,7 @@
         <v>35.75</v>
       </c>
       <c r="F849" t="n">
-        <v>20.5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="850">
@@ -17458,7 +17458,7 @@
         <v>27.5</v>
       </c>
       <c r="F851" t="n">
-        <v>13</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="852">
@@ -17478,7 +17478,7 @@
         <v>33.25</v>
       </c>
       <c r="F852" t="n">
-        <v>19</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="853">
@@ -17498,7 +17498,7 @@
         <v>26.5</v>
       </c>
       <c r="F853" t="n">
-        <v>20.5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="854">
@@ -17538,7 +17538,7 @@
         <v>-1.5</v>
       </c>
       <c r="F855" t="n">
-        <v>17.5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="856">
@@ -18178,7 +18178,7 @@
         <v>3.25</v>
       </c>
       <c r="F887" t="n">
-        <v>14.5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="888">
@@ -18258,7 +18258,7 @@
         <v>17.5</v>
       </c>
       <c r="F891" t="n">
-        <v>19</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="892">
@@ -18278,7 +18278,7 @@
         <v>20.5</v>
       </c>
       <c r="F892" t="n">
-        <v>17.5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="893">
@@ -18318,7 +18318,7 @@
         <v>37.75</v>
       </c>
       <c r="F894" t="n">
-        <v>14.5</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="895">
@@ -18338,7 +18338,7 @@
         <v>35.75</v>
       </c>
       <c r="F895" t="n">
-        <v>22</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="896">
@@ -18378,7 +18378,7 @@
         <v>35.25</v>
       </c>
       <c r="F897" t="n">
-        <v>20.5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="898">
@@ -18438,7 +18438,7 @@
         <v>35.25</v>
       </c>
       <c r="F900" t="n">
-        <v>14.5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="901">
@@ -18938,7 +18938,7 @@
         <v>25.75</v>
       </c>
       <c r="F925" t="n">
-        <v>20.5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="926">
@@ -19018,7 +19018,7 @@
         <v>35.75</v>
       </c>
       <c r="F929" t="n">
-        <v>22</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="930">
@@ -19598,7 +19598,7 @@
         <v>39.75</v>
       </c>
       <c r="F958" t="n">
-        <v>23.5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="959">
@@ -20658,7 +20658,7 @@
         <v>11.25</v>
       </c>
       <c r="F1011" t="n">
-        <v>19</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="1012">
@@ -20678,7 +20678,7 @@
         <v>35.25</v>
       </c>
       <c r="F1012" t="n">
-        <v>16</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="1013">
@@ -20738,7 +20738,7 @@
         <v>37.25</v>
       </c>
       <c r="F1015" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="1016">
@@ -21478,7 +21478,7 @@
         <v>34</v>
       </c>
       <c r="F1052" t="n">
-        <v>20.5</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="1053">
@@ -21518,7 +21518,7 @@
         <v>36.5</v>
       </c>
       <c r="F1054" t="n">
-        <v>23.5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="1055">
@@ -21538,7 +21538,7 @@
         <v>41.25</v>
       </c>
       <c r="F1055" t="n">
-        <v>22</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="1056">
@@ -26798,7 +26798,7 @@
         <v>25.25</v>
       </c>
       <c r="F1318" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="1319">
@@ -26818,7 +26818,7 @@
         <v>28</v>
       </c>
       <c r="F1319" t="n">
-        <v>23.5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="1320">
@@ -26838,7 +26838,7 @@
         <v>31.5</v>
       </c>
       <c r="F1320" t="n">
-        <v>20.5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="1321">
@@ -26878,7 +26878,7 @@
         <v>3.5</v>
       </c>
       <c r="F1322" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="1323">
@@ -26898,7 +26898,7 @@
         <v>24.75</v>
       </c>
       <c r="F1323" t="n">
-        <v>17.5</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="1324">
@@ -27298,7 +27298,7 @@
         <v>34.5</v>
       </c>
       <c r="F1343" t="n">
-        <v>22</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="1344">
@@ -27358,7 +27358,7 @@
         <v>36</v>
       </c>
       <c r="F1346" t="n">
-        <v>23.5</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="1347">
@@ -27478,7 +27478,7 @@
         <v>39.25</v>
       </c>
       <c r="F1352" t="n">
-        <v>17.5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="1353">
@@ -27818,7 +27818,7 @@
         <v>29.75</v>
       </c>
       <c r="F1369" t="n">
-        <v>20.5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="1370">
@@ -28898,7 +28898,7 @@
         <v>22.75</v>
       </c>
       <c r="F1423" t="n">
-        <v>20.5</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="1424">
@@ -28918,7 +28918,7 @@
         <v>39</v>
       </c>
       <c r="F1424" t="n">
-        <v>17.5</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="1425">
@@ -29078,7 +29078,7 @@
         <v>40.5</v>
       </c>
       <c r="F1432" t="n">
-        <v>22</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="1433">
@@ -29098,7 +29098,7 @@
         <v>38.5</v>
       </c>
       <c r="F1433" t="n">
-        <v>23.5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="1434">
@@ -29118,7 +29118,7 @@
         <v>42.5</v>
       </c>
       <c r="F1434" t="n">
-        <v>20.5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="1435">
@@ -30178,7 +30178,7 @@
         <v>43.25</v>
       </c>
       <c r="F1487" t="n">
-        <v>20.5</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="1488">
@@ -30198,7 +30198,7 @@
         <v>36.5</v>
       </c>
       <c r="F1488" t="n">
-        <v>23.5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="1489">
@@ -30398,7 +30398,7 @@
         <v>40.5</v>
       </c>
       <c r="F1498" t="n">
-        <v>20.5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="1499">
@@ -30543,7 +30543,7 @@
         <v>27.26</v>
       </c>
       <c r="F3" t="n">
-        <v>15.843</v>
+        <v>15.866</v>
       </c>
     </row>
     <row r="4">
@@ -30565,7 +30565,7 @@
         <v>14.51602424816504</v>
       </c>
       <c r="F4" t="n">
-        <v>9.101377609072214</v>
+        <v>9.110564138366042</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
reorganizacion del directorio ./analysis/
</commit_message>
<xml_diff>
--- a/results/logs/episode_rewards.xlsx
+++ b/results/logs/episode_rewards.xlsx
@@ -459,10 +459,10 @@
         <v>148</v>
       </c>
       <c r="C2" t="n">
-        <v>-115.255559837265</v>
+        <v>-131.5339542548244</v>
       </c>
       <c r="D2" t="n">
-        <v>76</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -522,10 +522,10 @@
         <v>148</v>
       </c>
       <c r="C3" t="n">
-        <v>-115.255559837265</v>
+        <v>-131.5339542548244</v>
       </c>
       <c r="D3" t="n">
-        <v>76</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4">
@@ -548,10 +548,10 @@
         <v>148</v>
       </c>
       <c r="C5" t="n">
-        <v>-115.255559837265</v>
+        <v>-131.5339542548244</v>
       </c>
       <c r="D5" t="n">
-        <v>76</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6">
@@ -564,10 +564,10 @@
         <v>148</v>
       </c>
       <c r="C6" t="n">
-        <v>-115.255559837265</v>
+        <v>-131.5339542548244</v>
       </c>
       <c r="D6" t="n">
-        <v>76</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7">
@@ -580,10 +580,10 @@
         <v>148</v>
       </c>
       <c r="C7" t="n">
-        <v>-115.255559837265</v>
+        <v>-131.5339542548244</v>
       </c>
       <c r="D7" t="n">
-        <v>76</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8">
@@ -596,10 +596,10 @@
         <v>148</v>
       </c>
       <c r="C8" t="n">
-        <v>-115.255559837265</v>
+        <v>-131.5339542548244</v>
       </c>
       <c r="D8" t="n">
-        <v>76</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9">
@@ -612,10 +612,10 @@
         <v>148</v>
       </c>
       <c r="C9" t="n">
-        <v>-115.255559837265</v>
+        <v>-131.5339542548244</v>
       </c>
       <c r="D9" t="n">
-        <v>76</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>